<commit_message>
atualização dos dados de 2Q26
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/micron/mu_indicators.xlsx
+++ b/analise_eua/semicondutores/micron/mu_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,168 +436,170 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
         <v>21.85</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>21.85</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.58</v>
+      </c>
       <c r="E2" t="n">
         <v>18122</v>
       </c>
@@ -591,7 +607,7 @@
         <v>22.84</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>3.44</v>
       </c>
       <c r="H2" t="n">
         <v>186539400</v>
@@ -667,16 +683,18 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
         <v>146.46</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>147.31</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.68</v>
+      </c>
       <c r="E3" t="n">
         <v>9084</v>
       </c>
@@ -684,7 +702,7 @@
         <v>3.1</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2.52</v>
       </c>
       <c r="H3" t="n">
         <v>113947600</v>
@@ -760,7 +778,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B4" t="n">
@@ -769,7 +787,9 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>-7.93</v>
+      </c>
       <c r="E4" t="n">
         <v>2011</v>
       </c>
@@ -777,7 +797,7 @@
         <v>-37.54</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H4" t="n">
         <v>73580760</v>
@@ -853,16 +873,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B5" t="n">
         <v>6.29</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>6.3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15.88</v>
+      </c>
       <c r="E5" t="n">
         <v>16818</v>
       </c>
@@ -870,7 +892,7 @@
         <v>28.24</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="H5" t="n">
         <v>54677040</v>
@@ -946,16 +968,18 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="B6" t="n">
         <v>13.25</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>13.26</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7.54</v>
+      </c>
       <c r="E6" t="n">
         <v>12497</v>
       </c>
@@ -963,7 +987,7 @@
         <v>21.16</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1.77</v>
       </c>
       <c r="H6" t="n">
         <v>77672000</v>
@@ -1039,16 +1063,18 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="B7" t="n">
         <v>18.93</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>18.93</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.28</v>
+      </c>
       <c r="E7" t="n">
         <v>8653</v>
       </c>
@@ -1056,7 +1082,7 @@
         <v>12.54</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="H7" t="n">
         <v>50860200</v>
@@ -1132,16 +1158,18 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="B8" t="n">
         <v>7.38</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr"/>
+        <v>7.37</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13.56</v>
+      </c>
       <c r="E8" t="n">
         <v>12800</v>
       </c>
@@ -1149,7 +1177,7 @@
         <v>26.97</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="H8" t="n">
         <v>46576340.00000001</v>
@@ -1225,16 +1253,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="B9" t="n">
         <v>3.6</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>3.6</v>
+      </c>
+      <c r="D9" t="n">
+        <v>27.8</v>
+      </c>
       <c r="E9" t="n">
         <v>19753</v>
       </c>
@@ -1242,7 +1272,7 @@
         <v>46.51</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1.57</v>
       </c>
       <c r="H9" t="n">
         <v>50837760</v>
@@ -1318,16 +1348,18 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>2017</v>
       </c>
       <c r="B10" t="n">
         <v>8.210000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>8.220000000000001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12.17</v>
+      </c>
       <c r="E10" t="n">
         <v>9729</v>
       </c>
@@ -1335,7 +1367,7 @@
         <v>25.04</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>2.24</v>
       </c>
       <c r="H10" t="n">
         <v>41784930</v>
@@ -1421,1575 +1453,1575 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46018</v>
+      <c r="A2" s="2" t="n">
+        <v>46107</v>
       </c>
       <c r="B2" t="n">
-        <v>61.28</v>
+        <v>29.04</v>
       </c>
       <c r="C2" t="n">
-        <v>30.2</v>
+        <v>17.76</v>
       </c>
       <c r="D2" t="n">
-        <v>3.31</v>
+        <v>5.63</v>
       </c>
       <c r="E2" t="n">
-        <v>8348</v>
+        <v>18421</v>
       </c>
       <c r="F2" t="n">
-        <v>38.41</v>
+        <v>57.77</v>
       </c>
       <c r="G2" t="n">
-        <v>5.46</v>
+        <v>5.52</v>
       </c>
       <c r="H2" t="n">
-        <v>321086250</v>
+        <v>400247959.9999999</v>
       </c>
       <c r="I2" t="n">
-        <v>12425</v>
+        <v>10798</v>
       </c>
       <c r="J2" t="n">
-        <v>10318</v>
+        <v>14589</v>
       </c>
       <c r="K2" t="n">
-        <v>2107</v>
+        <v>-3791</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="M2" t="n">
-        <v>0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="N2" t="n">
-        <v>15.64</v>
+        <v>11.58</v>
       </c>
       <c r="O2" t="n">
-        <v>17.99</v>
+        <v>31.04</v>
       </c>
       <c r="P2" t="n">
-        <v>19.34</v>
+        <v>35.82</v>
       </c>
       <c r="Q2" t="n">
-        <v>8411</v>
+        <v>11903</v>
       </c>
       <c r="R2" t="n">
-        <v>-4594</v>
+        <v>-5525</v>
       </c>
       <c r="S2" t="n">
-        <v>-3745</v>
+        <v>-2167</v>
       </c>
       <c r="T2" t="n">
-        <v>3022</v>
+        <v>5516</v>
       </c>
       <c r="U2" t="n">
-        <v>5389</v>
+        <v>6387</v>
       </c>
       <c r="V2" t="n">
-        <v>7173</v>
+        <v>10098</v>
       </c>
       <c r="W2" t="n">
-        <v>1171</v>
+        <v>1250</v>
       </c>
       <c r="X2" t="n">
-        <v>11095</v>
+        <v>14382</v>
       </c>
       <c r="Y2" t="n">
-        <v>17605</v>
+        <v>27117</v>
       </c>
       <c r="Z2" t="n">
-        <v>81.38</v>
+        <v>67.32000000000001</v>
       </c>
       <c r="AA2" t="n">
-        <v>1172</v>
+        <v>2982</v>
       </c>
       <c r="AB2" t="n">
-        <v>4963</v>
+        <v>10418</v>
       </c>
       <c r="AC2" t="n">
         <v>0.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>2.56</v>
+        <v>0.96</v>
       </c>
       <c r="AE2" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45837</v>
+      <c r="A3" s="2" t="n">
+        <v>46018</v>
       </c>
       <c r="B3" t="n">
-        <v>72.95999999999999</v>
+        <v>61.28</v>
       </c>
       <c r="C3" t="n">
-        <v>24.17</v>
+        <v>30.2</v>
       </c>
       <c r="D3" t="n">
-        <v>4.14</v>
+        <v>3.31</v>
       </c>
       <c r="E3" t="n">
-        <v>4263</v>
+        <v>8348</v>
       </c>
       <c r="F3" t="n">
-        <v>20.27</v>
+        <v>38.41</v>
       </c>
       <c r="G3" t="n">
-        <v>2.71</v>
+        <v>5.46</v>
       </c>
       <c r="H3" t="n">
-        <v>137525180</v>
+        <v>321086250</v>
       </c>
       <c r="I3" t="n">
-        <v>16141</v>
+        <v>12425</v>
       </c>
       <c r="J3" t="n">
-        <v>10811</v>
+        <v>10318</v>
       </c>
       <c r="K3" t="n">
-        <v>5330</v>
+        <v>2107</v>
       </c>
       <c r="L3" t="n">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="M3" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="N3" t="n">
-        <v>9.529999999999999</v>
+        <v>15.64</v>
       </c>
       <c r="O3" t="n">
-        <v>11.17</v>
+        <v>17.99</v>
       </c>
       <c r="P3" t="n">
-        <v>11.82</v>
+        <v>19.34</v>
       </c>
       <c r="Q3" t="n">
-        <v>4609</v>
+        <v>8411</v>
       </c>
       <c r="R3" t="n">
-        <v>-2589</v>
+        <v>-4594</v>
       </c>
       <c r="S3" t="n">
-        <v>540</v>
+        <v>-3745</v>
       </c>
       <c r="T3" t="n">
-        <v>1671</v>
+        <v>3022</v>
       </c>
       <c r="U3" t="n">
-        <v>2938</v>
+        <v>5389</v>
       </c>
       <c r="V3" t="n">
-        <v>4127</v>
+        <v>7173</v>
       </c>
       <c r="W3" t="n">
-        <v>965</v>
+        <v>1171</v>
       </c>
       <c r="X3" t="n">
-        <v>7728</v>
+        <v>11095</v>
       </c>
       <c r="Y3" t="n">
-        <v>17784</v>
+        <v>17605</v>
       </c>
       <c r="Z3" t="n">
-        <v>95.09</v>
+        <v>81.38</v>
       </c>
       <c r="AA3" t="n">
-        <v>1863</v>
+        <v>1172</v>
       </c>
       <c r="AB3" t="n">
-        <v>2917</v>
+        <v>4963</v>
       </c>
       <c r="AC3" t="n">
         <v>0.12</v>
       </c>
       <c r="AD3" t="n">
-        <v>6.95</v>
+        <v>2.56</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45743</v>
+      <c r="A4" s="2" t="n">
+        <v>45837</v>
       </c>
       <c r="B4" t="n">
-        <v>61.08</v>
+        <v>72.95999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>21.05</v>
+        <v>24.17</v>
       </c>
       <c r="D4" t="n">
-        <v>4.75</v>
+        <v>4.14</v>
       </c>
       <c r="E4" t="n">
-        <v>3852</v>
+        <v>4263</v>
       </c>
       <c r="F4" t="n">
-        <v>19.66</v>
+        <v>20.27</v>
       </c>
       <c r="G4" t="n">
-        <v>1.99</v>
+        <v>2.71</v>
       </c>
       <c r="H4" t="n">
-        <v>96692800</v>
+        <v>137525180</v>
       </c>
       <c r="I4" t="n">
-        <v>14954</v>
+        <v>16141</v>
       </c>
       <c r="J4" t="n">
-        <v>8215</v>
+        <v>10811</v>
       </c>
       <c r="K4" t="n">
-        <v>6739</v>
+        <v>5330</v>
       </c>
       <c r="L4" t="n">
-        <v>0.52</v>
+        <v>0.36</v>
       </c>
       <c r="M4" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="N4" t="n">
-        <v>8.050000000000001</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="O4" t="n">
-        <v>9.41</v>
+        <v>11.17</v>
       </c>
       <c r="P4" t="n">
-        <v>7.98</v>
+        <v>11.82</v>
       </c>
       <c r="Q4" t="n">
-        <v>3942</v>
+        <v>4609</v>
       </c>
       <c r="R4" t="n">
-        <v>-3152</v>
+        <v>-2589</v>
       </c>
       <c r="S4" t="n">
-        <v>96</v>
+        <v>540</v>
       </c>
       <c r="T4" t="n">
-        <v>-113</v>
+        <v>1671</v>
       </c>
       <c r="U4" t="n">
-        <v>4055</v>
+        <v>2938</v>
       </c>
       <c r="V4" t="n">
-        <v>2743</v>
+        <v>4127</v>
       </c>
       <c r="W4" t="n">
-        <v>898</v>
+        <v>965</v>
       </c>
       <c r="X4" t="n">
-        <v>6211</v>
+        <v>7728</v>
       </c>
       <c r="Y4" t="n">
-        <v>16812</v>
+        <v>17784</v>
       </c>
       <c r="Z4" t="n">
-        <v>122.14</v>
+        <v>95.09</v>
       </c>
       <c r="AA4" t="n">
-        <v>1143</v>
+        <v>1863</v>
       </c>
       <c r="AB4" t="n">
-        <v>2130</v>
+        <v>2917</v>
       </c>
       <c r="AC4" t="n">
         <v>0.12</v>
       </c>
       <c r="AD4" t="n">
-        <v>8.210000000000001</v>
+        <v>6.95</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45654</v>
+      <c r="A5" s="2" t="n">
+        <v>45743</v>
       </c>
       <c r="B5" t="n">
-        <v>49.84</v>
+        <v>61.08</v>
       </c>
       <c r="C5" t="n">
-        <v>53.09</v>
+        <v>21.05</v>
       </c>
       <c r="D5" t="n">
-        <v>1.88</v>
+        <v>4.75</v>
       </c>
       <c r="E5" t="n">
-        <v>4204</v>
+        <v>3852</v>
       </c>
       <c r="F5" t="n">
-        <v>21.47</v>
+        <v>19.66</v>
       </c>
       <c r="G5" t="n">
         <v>1.99</v>
       </c>
       <c r="H5" t="n">
-        <v>93201790</v>
+        <v>96692800</v>
       </c>
       <c r="I5" t="n">
-        <v>14373</v>
+        <v>14954</v>
       </c>
       <c r="J5" t="n">
-        <v>7588</v>
+        <v>8215</v>
       </c>
       <c r="K5" t="n">
-        <v>6785</v>
+        <v>6739</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="M5" t="n">
         <v>0.14</v>
       </c>
       <c r="N5" t="n">
-        <v>10.22</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="O5" t="n">
-        <v>3.76</v>
+        <v>9.41</v>
       </c>
       <c r="P5" t="n">
-        <v>3.38</v>
+        <v>7.98</v>
       </c>
       <c r="Q5" t="n">
-        <v>3244</v>
+        <v>3942</v>
       </c>
       <c r="R5" t="n">
-        <v>-3148</v>
+        <v>-3152</v>
       </c>
       <c r="S5" t="n">
-        <v>-422</v>
+        <v>96</v>
       </c>
       <c r="T5" t="n">
-        <v>38</v>
+        <v>-113</v>
       </c>
       <c r="U5" t="n">
-        <v>3206</v>
+        <v>4055</v>
       </c>
       <c r="V5" t="n">
-        <v>648</v>
+        <v>2743</v>
       </c>
       <c r="W5" t="n">
-        <v>888</v>
+        <v>898</v>
       </c>
       <c r="X5" t="n">
-        <v>4063</v>
+        <v>6211</v>
       </c>
       <c r="Y5" t="n">
-        <v>15478</v>
+        <v>16812</v>
       </c>
       <c r="Z5" t="n">
-        <v>247.31</v>
+        <v>122.14</v>
       </c>
       <c r="AA5" t="n">
-        <v>-837</v>
+        <v>1143</v>
       </c>
       <c r="AB5" t="n">
-        <v>259</v>
+        <v>2130</v>
       </c>
       <c r="AC5" t="n">
         <v>0.12</v>
       </c>
       <c r="AD5" t="n">
-        <v>7.01</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45473</v>
+      <c r="A6" s="2" t="n">
+        <v>45654</v>
       </c>
       <c r="B6" t="n">
-        <v>435.7</v>
+        <v>49.84</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>53.09</v>
       </c>
       <c r="D6" t="n">
-        <v>-1.4</v>
+        <v>1.88</v>
       </c>
       <c r="E6" t="n">
-        <v>2674</v>
+        <v>4204</v>
       </c>
       <c r="F6" t="n">
-        <v>4.87</v>
+        <v>21.47</v>
       </c>
       <c r="G6" t="n">
-        <v>3.27</v>
+        <v>1.99</v>
       </c>
       <c r="H6" t="n">
-        <v>144651690</v>
+        <v>93201790</v>
       </c>
       <c r="I6" t="n">
-        <v>13867</v>
+        <v>14373</v>
       </c>
       <c r="J6" t="n">
-        <v>8379</v>
+        <v>7588</v>
       </c>
       <c r="K6" t="n">
-        <v>5488</v>
+        <v>6785</v>
       </c>
       <c r="L6" t="n">
-        <v>0.95</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="N6" t="n">
-        <v>26.02</v>
+        <v>10.22</v>
       </c>
       <c r="O6" t="n">
-        <v>-4.53</v>
+        <v>3.76</v>
       </c>
       <c r="P6" t="n">
-        <v>-3.46</v>
+        <v>3.38</v>
       </c>
       <c r="Q6" t="n">
-        <v>2482</v>
+        <v>3244</v>
       </c>
       <c r="R6" t="n">
-        <v>-2002</v>
+        <v>-3148</v>
       </c>
       <c r="S6" t="n">
-        <v>-910</v>
+        <v>-422</v>
       </c>
       <c r="T6" t="n">
-        <v>396</v>
+        <v>38</v>
       </c>
       <c r="U6" t="n">
-        <v>2086</v>
+        <v>3206</v>
       </c>
       <c r="V6" t="n">
-        <v>-923</v>
+        <v>648</v>
       </c>
       <c r="W6" t="n">
-        <v>850</v>
+        <v>888</v>
       </c>
       <c r="X6" t="n">
-        <v>2362</v>
+        <v>4063</v>
       </c>
       <c r="Y6" t="n">
-        <v>16479</v>
+        <v>15478</v>
       </c>
       <c r="Z6" t="n">
-        <v>-125.89</v>
+        <v>247.31</v>
       </c>
       <c r="AA6" t="n">
-        <v>-1228</v>
+        <v>-837</v>
       </c>
       <c r="AB6" t="n">
-        <v>-2270</v>
+        <v>259</v>
       </c>
       <c r="AC6" t="n">
         <v>0.12</v>
       </c>
       <c r="AD6" t="n">
-        <v>38.55</v>
+        <v>7.01</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45380</v>
+      <c r="A7" s="2" t="n">
+        <v>45473</v>
       </c>
       <c r="B7" t="n">
-        <v>163.05</v>
+        <v>435.7</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>-3.63</v>
+        <v>-1.4</v>
       </c>
       <c r="E7" t="n">
-        <v>2115</v>
+        <v>2674</v>
       </c>
       <c r="F7" t="n">
-        <v>13.62</v>
+        <v>4.87</v>
       </c>
       <c r="G7" t="n">
-        <v>2.95</v>
+        <v>3.27</v>
       </c>
       <c r="H7" t="n">
-        <v>129300480</v>
+        <v>144651690</v>
       </c>
       <c r="I7" t="n">
-        <v>14315</v>
+        <v>13867</v>
       </c>
       <c r="J7" t="n">
-        <v>9006</v>
+        <v>8379</v>
       </c>
       <c r="K7" t="n">
-        <v>5309</v>
+        <v>5488</v>
       </c>
       <c r="L7" t="n">
-        <v>1.94</v>
+        <v>0.95</v>
       </c>
       <c r="M7" t="n">
         <v>0.12</v>
       </c>
       <c r="N7" t="n">
-        <v>49.2</v>
+        <v>26.02</v>
       </c>
       <c r="O7" t="n">
-        <v>-10.6</v>
+        <v>-4.53</v>
       </c>
       <c r="P7" t="n">
-        <v>-9.210000000000001</v>
+        <v>-3.46</v>
       </c>
       <c r="Q7" t="n">
-        <v>1219</v>
+        <v>2482</v>
       </c>
       <c r="R7" t="n">
-        <v>-1151</v>
+        <v>-2002</v>
       </c>
       <c r="S7" t="n">
-        <v>-106</v>
+        <v>-910</v>
       </c>
       <c r="T7" t="n">
-        <v>-165</v>
+        <v>396</v>
       </c>
       <c r="U7" t="n">
-        <v>1384</v>
+        <v>2086</v>
       </c>
       <c r="V7" t="n">
-        <v>-791</v>
+        <v>-923</v>
       </c>
       <c r="W7" t="n">
-        <v>832</v>
+        <v>850</v>
       </c>
       <c r="X7" t="n">
-        <v>2432</v>
+        <v>2362</v>
       </c>
       <c r="Y7" t="n">
-        <v>17176</v>
+        <v>16479</v>
       </c>
       <c r="Z7" t="n">
-        <v>-78.92</v>
+        <v>-125.89</v>
       </c>
       <c r="AA7" t="n">
-        <v>-3075</v>
+        <v>-1228</v>
       </c>
       <c r="AB7" t="n">
-        <v>-6006</v>
+        <v>-2270</v>
       </c>
       <c r="AC7" t="n">
         <v>0.12</v>
       </c>
       <c r="AD7" t="n">
-        <v>16.02</v>
+        <v>38.55</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45290</v>
+      <c r="A8" s="2" t="n">
+        <v>45380</v>
       </c>
       <c r="B8" t="n">
-        <v>-75.5</v>
+        <v>163.05</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>-6.08</v>
+        <v>-3.63</v>
       </c>
       <c r="E8" t="n">
-        <v>787</v>
+        <v>2115</v>
       </c>
       <c r="F8" t="n">
-        <v>-26.11</v>
+        <v>13.62</v>
       </c>
       <c r="G8" t="n">
-        <v>2.17</v>
+        <v>2.95</v>
       </c>
       <c r="H8" t="n">
-        <v>93170000</v>
+        <v>129300480</v>
       </c>
       <c r="I8" t="n">
-        <v>14106</v>
+        <v>14315</v>
       </c>
       <c r="J8" t="n">
-        <v>9048</v>
+        <v>9006</v>
       </c>
       <c r="K8" t="n">
-        <v>5058</v>
+        <v>5309</v>
       </c>
       <c r="L8" t="n">
-        <v>2.17</v>
+        <v>1.94</v>
       </c>
       <c r="M8" t="n">
         <v>0.12</v>
       </c>
       <c r="N8" t="n">
-        <v>42.1</v>
+        <v>49.2</v>
       </c>
       <c r="O8" t="n">
-        <v>-13.14</v>
+        <v>-10.6</v>
       </c>
       <c r="P8" t="n">
-        <v>-9</v>
+        <v>-9.210000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>1401</v>
+        <v>1219</v>
       </c>
       <c r="R8" t="n">
-        <v>-1558</v>
+        <v>-1151</v>
       </c>
       <c r="S8" t="n">
-        <v>-352</v>
+        <v>-106</v>
       </c>
       <c r="T8" t="n">
-        <v>-395</v>
+        <v>-165</v>
       </c>
       <c r="U8" t="n">
-        <v>1796</v>
+        <v>1384</v>
       </c>
       <c r="V8" t="n">
-        <v>277</v>
+        <v>-791</v>
       </c>
       <c r="W8" t="n">
-        <v>845</v>
+        <v>832</v>
       </c>
       <c r="X8" t="n">
-        <v>3517</v>
+        <v>2432</v>
       </c>
       <c r="Y8" t="n">
-        <v>15096</v>
+        <v>17176</v>
       </c>
       <c r="Z8" t="n">
-        <v>-59.63</v>
+        <v>-78.92</v>
       </c>
       <c r="AA8" t="n">
-        <v>503</v>
+        <v>-3075</v>
       </c>
       <c r="AB8" t="n">
-        <v>-5218</v>
+        <v>-6006</v>
       </c>
       <c r="AC8" t="n">
         <v>0.12</v>
       </c>
       <c r="AD8" t="n">
-        <v>-10.45</v>
+        <v>16.02</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45078</v>
+      <c r="A9" s="2" t="n">
+        <v>45290</v>
       </c>
       <c r="B9" t="n">
-        <v>-35.96</v>
+        <v>-75.5</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-2.68</v>
+        <v>-6.08</v>
       </c>
       <c r="E9" t="n">
-        <v>195</v>
+        <v>787</v>
       </c>
       <c r="F9" t="n">
-        <v>-50.53</v>
+        <v>-26.11</v>
       </c>
       <c r="G9" t="n">
-        <v>1.5</v>
+        <v>2.17</v>
       </c>
       <c r="H9" t="n">
-        <v>68189020</v>
+        <v>93170000</v>
       </c>
       <c r="I9" t="n">
-        <v>13848</v>
+        <v>14106</v>
       </c>
       <c r="J9" t="n">
-        <v>10352</v>
+        <v>9048</v>
       </c>
       <c r="K9" t="n">
-        <v>3496</v>
+        <v>5058</v>
       </c>
       <c r="L9" t="n">
-        <v>0.55</v>
+        <v>2.17</v>
       </c>
       <c r="M9" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="N9" t="n">
-        <v>11.25</v>
+        <v>42.1</v>
       </c>
       <c r="O9" t="n">
-        <v>-3.91</v>
+        <v>-13.14</v>
       </c>
       <c r="P9" t="n">
-        <v>-1.2</v>
+        <v>-9</v>
       </c>
       <c r="Q9" t="n">
-        <v>24</v>
+        <v>1401</v>
       </c>
       <c r="R9" t="n">
-        <v>-1180</v>
+        <v>-1558</v>
       </c>
       <c r="S9" t="n">
-        <v>661</v>
+        <v>-352</v>
       </c>
       <c r="T9" t="n">
-        <v>-1537</v>
+        <v>-395</v>
       </c>
       <c r="U9" t="n">
-        <v>1561</v>
+        <v>1796</v>
       </c>
       <c r="V9" t="n">
-        <v>1153</v>
+        <v>277</v>
       </c>
       <c r="W9" t="n">
-        <v>758</v>
+        <v>845</v>
       </c>
       <c r="X9" t="n">
-        <v>4321</v>
+        <v>3517</v>
       </c>
       <c r="Y9" t="n">
-        <v>16630</v>
+        <v>15096</v>
       </c>
       <c r="Z9" t="n">
-        <v>-701.6899999999999</v>
+        <v>-59.63</v>
       </c>
       <c r="AA9" t="n">
-        <v>2392</v>
+        <v>503</v>
       </c>
       <c r="AB9" t="n">
-        <v>-3083</v>
+        <v>-5218</v>
       </c>
       <c r="AC9" t="n">
         <v>0.12</v>
       </c>
       <c r="AD9" t="n">
-        <v>-6.65</v>
+        <v>-10.45</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>44987</v>
+      <c r="A10" s="2" t="n">
+        <v>45078</v>
       </c>
       <c r="B10" t="n">
-        <v>-28.07</v>
+        <v>-35.96</v>
       </c>
       <c r="C10" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>3.5</v>
+        <v>-2.68</v>
       </c>
       <c r="E10" t="n">
-        <v>-361</v>
+        <v>195</v>
       </c>
       <c r="F10" t="n">
-        <v>-62.6</v>
+        <v>-50.53</v>
       </c>
       <c r="G10" t="n">
-        <v>1.37</v>
+        <v>1.5</v>
       </c>
       <c r="H10" t="n">
-        <v>64892679.99999999</v>
+        <v>68189020</v>
       </c>
       <c r="I10" t="n">
-        <v>12884</v>
+        <v>13848</v>
       </c>
       <c r="J10" t="n">
-        <v>10818</v>
+        <v>10352</v>
       </c>
       <c r="K10" t="n">
-        <v>2066</v>
+        <v>3496</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2</v>
+        <v>0.55</v>
       </c>
       <c r="M10" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="N10" t="n">
-        <v>6.4</v>
+        <v>11.25</v>
       </c>
       <c r="O10" t="n">
-        <v>5.04</v>
+        <v>-3.91</v>
       </c>
       <c r="P10" t="n">
-        <v>6.17</v>
+        <v>-1.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>343</v>
+        <v>24</v>
       </c>
       <c r="R10" t="n">
-        <v>-1915</v>
+        <v>-1180</v>
       </c>
       <c r="S10" t="n">
-        <v>1802</v>
+        <v>661</v>
       </c>
       <c r="T10" t="n">
-        <v>-1862</v>
+        <v>-1537</v>
       </c>
       <c r="U10" t="n">
-        <v>2205</v>
+        <v>1561</v>
       </c>
       <c r="V10" t="n">
-        <v>2417</v>
+        <v>1153</v>
       </c>
       <c r="W10" t="n">
-        <v>788</v>
+        <v>758</v>
       </c>
       <c r="X10" t="n">
-        <v>5619</v>
+        <v>4321</v>
       </c>
       <c r="Y10" t="n">
-        <v>16643</v>
+        <v>16630</v>
       </c>
       <c r="Z10" t="n">
-        <v>174.76</v>
+        <v>-701.6899999999999</v>
       </c>
       <c r="AA10" t="n">
-        <v>4204</v>
+        <v>2392</v>
       </c>
       <c r="AB10" t="n">
-        <v>-321</v>
+        <v>-3083</v>
       </c>
       <c r="AC10" t="n">
         <v>0.12</v>
       </c>
       <c r="AD10" t="n">
-        <v>-5.45</v>
+        <v>-6.65</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>44896</v>
+      <c r="A11" s="2" t="n">
+        <v>44987</v>
       </c>
       <c r="B11" t="n">
-        <v>-275.35</v>
+        <v>-28.07</v>
       </c>
       <c r="C11" t="n">
-        <v>7.87</v>
+        <v>28.6</v>
       </c>
       <c r="D11" t="n">
-        <v>12.71</v>
+        <v>3.5</v>
       </c>
       <c r="E11" t="n">
-        <v>1712</v>
+        <v>-361</v>
       </c>
       <c r="F11" t="n">
-        <v>-4.77</v>
+        <v>-62.6</v>
       </c>
       <c r="G11" t="n">
-        <v>1.09</v>
+        <v>1.37</v>
       </c>
       <c r="H11" t="n">
-        <v>53693400</v>
+        <v>64892679.99999999</v>
       </c>
       <c r="I11" t="n">
-        <v>10890</v>
+        <v>12884</v>
       </c>
       <c r="J11" t="n">
-        <v>10581</v>
+        <v>10818</v>
       </c>
       <c r="K11" t="n">
-        <v>309</v>
+        <v>2066</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="M11" t="n">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="N11" t="n">
-        <v>3.57</v>
+        <v>6.4</v>
       </c>
       <c r="O11" t="n">
-        <v>14.2</v>
+        <v>5.04</v>
       </c>
       <c r="P11" t="n">
-        <v>14.64</v>
+        <v>6.17</v>
       </c>
       <c r="Q11" t="n">
-        <v>943</v>
+        <v>343</v>
       </c>
       <c r="R11" t="n">
-        <v>-2266</v>
+        <v>-1915</v>
       </c>
       <c r="S11" t="n">
-        <v>2632</v>
+        <v>1802</v>
       </c>
       <c r="T11" t="n">
-        <v>-1506</v>
+        <v>-1862</v>
       </c>
       <c r="U11" t="n">
-        <v>2449</v>
+        <v>2205</v>
       </c>
       <c r="V11" t="n">
-        <v>3748</v>
+        <v>2417</v>
       </c>
       <c r="W11" t="n">
-        <v>849</v>
+        <v>788</v>
       </c>
       <c r="X11" t="n">
-        <v>6874</v>
+        <v>5619</v>
       </c>
       <c r="Y11" t="n">
-        <v>16396</v>
+        <v>16643</v>
       </c>
       <c r="Z11" t="n">
-        <v>88.34999999999999</v>
+        <v>174.76</v>
       </c>
       <c r="AA11" t="n">
-        <v>5662</v>
+        <v>4204</v>
       </c>
       <c r="AB11" t="n">
-        <v>2951</v>
+        <v>-321</v>
       </c>
       <c r="AC11" t="n">
         <v>0.12</v>
       </c>
       <c r="AD11" t="n">
-        <v>-64.62</v>
+        <v>-5.45</v>
       </c>
       <c r="AE11" t="n">
-        <v>425</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>44714</v>
+      <c r="A12" s="2" t="n">
+        <v>44896</v>
       </c>
       <c r="B12" t="n">
-        <v>22.93</v>
+        <v>-275.35</v>
       </c>
       <c r="C12" t="n">
-        <v>6.78</v>
+        <v>7.87</v>
       </c>
       <c r="D12" t="n">
-        <v>14.76</v>
+        <v>12.71</v>
       </c>
       <c r="E12" t="n">
-        <v>4825</v>
+        <v>1712</v>
       </c>
       <c r="F12" t="n">
-        <v>30.39</v>
+        <v>-4.77</v>
       </c>
       <c r="G12" t="n">
-        <v>1.22</v>
+        <v>1.09</v>
       </c>
       <c r="H12" t="n">
-        <v>60203680</v>
+        <v>53693400</v>
       </c>
       <c r="I12" t="n">
-        <v>7592</v>
+        <v>10890</v>
       </c>
       <c r="J12" t="n">
-        <v>10227</v>
+        <v>10581</v>
       </c>
       <c r="K12" t="n">
-        <v>-2635</v>
+        <v>309</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.16</v>
+        <v>0.02</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.05</v>
+        <v>0.01</v>
       </c>
       <c r="N12" t="n">
-        <v>3.75</v>
+        <v>3.57</v>
       </c>
       <c r="O12" t="n">
-        <v>18.12</v>
+        <v>14.2</v>
       </c>
       <c r="P12" t="n">
-        <v>19.13</v>
+        <v>14.64</v>
       </c>
       <c r="Q12" t="n">
-        <v>3838</v>
+        <v>943</v>
       </c>
       <c r="R12" t="n">
-        <v>-2585</v>
+        <v>-2266</v>
       </c>
       <c r="S12" t="n">
-        <v>-1161</v>
+        <v>2632</v>
       </c>
       <c r="T12" t="n">
-        <v>1260</v>
+        <v>-1506</v>
       </c>
       <c r="U12" t="n">
-        <v>2578</v>
+        <v>2449</v>
       </c>
       <c r="V12" t="n">
-        <v>3922</v>
+        <v>3748</v>
       </c>
       <c r="W12" t="n">
-        <v>773</v>
+        <v>849</v>
       </c>
       <c r="X12" t="n">
-        <v>6869</v>
+        <v>6874</v>
       </c>
       <c r="Y12" t="n">
-        <v>15699</v>
+        <v>16396</v>
       </c>
       <c r="Z12" t="n">
-        <v>70.81</v>
+        <v>88.34999999999999</v>
       </c>
       <c r="AA12" t="n">
-        <v>4114</v>
+        <v>5662</v>
       </c>
       <c r="AB12" t="n">
-        <v>5225</v>
+        <v>2951</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="AD12" t="n">
-        <v>4.23</v>
+        <v>-64.62</v>
       </c>
       <c r="AE12" t="n">
-        <v>981</v>
+        <v>425</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>44623</v>
+      <c r="A13" s="2" t="n">
+        <v>44714</v>
       </c>
       <c r="B13" t="n">
-        <v>37.67</v>
+        <v>22.93</v>
       </c>
       <c r="C13" t="n">
-        <v>12.35</v>
+        <v>6.78</v>
       </c>
       <c r="D13" t="n">
-        <v>8.1</v>
+        <v>14.76</v>
       </c>
       <c r="E13" t="n">
-        <v>4288</v>
+        <v>4825</v>
       </c>
       <c r="F13" t="n">
-        <v>29.06</v>
+        <v>30.39</v>
       </c>
       <c r="G13" t="n">
-        <v>1.78</v>
+        <v>1.22</v>
       </c>
       <c r="H13" t="n">
-        <v>85245420.00000001</v>
+        <v>60203680</v>
       </c>
       <c r="I13" t="n">
-        <v>7611</v>
+        <v>7592</v>
       </c>
       <c r="J13" t="n">
-        <v>10122</v>
+        <v>10227</v>
       </c>
       <c r="K13" t="n">
-        <v>-2511</v>
+        <v>-2635</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.18</v>
+        <v>-0.16</v>
       </c>
       <c r="M13" t="n">
         <v>-0.05</v>
       </c>
       <c r="N13" t="n">
-        <v>6.2</v>
+        <v>3.75</v>
       </c>
       <c r="O13" t="n">
-        <v>14.44</v>
+        <v>18.12</v>
       </c>
       <c r="P13" t="n">
-        <v>14.83</v>
+        <v>19.13</v>
       </c>
       <c r="Q13" t="n">
-        <v>3628</v>
+        <v>3838</v>
       </c>
       <c r="R13" t="n">
-        <v>-2691</v>
+        <v>-2585</v>
       </c>
       <c r="S13" t="n">
-        <v>-466</v>
+        <v>-1161</v>
       </c>
       <c r="T13" t="n">
-        <v>1017</v>
+        <v>1260</v>
       </c>
       <c r="U13" t="n">
-        <v>2611</v>
+        <v>2578</v>
       </c>
       <c r="V13" t="n">
-        <v>4634</v>
+        <v>3922</v>
       </c>
       <c r="W13" t="n">
-        <v>792</v>
+        <v>773</v>
       </c>
       <c r="X13" t="n">
-        <v>7449</v>
+        <v>6869</v>
       </c>
       <c r="Y13" t="n">
-        <v>14584</v>
+        <v>15699</v>
       </c>
       <c r="Z13" t="n">
-        <v>96.85000000000001</v>
+        <v>70.81</v>
       </c>
       <c r="AA13" t="n">
-        <v>1702</v>
+        <v>4114</v>
       </c>
       <c r="AB13" t="n">
-        <v>2487</v>
+        <v>5225</v>
       </c>
       <c r="AC13" t="n">
         <v>0.1</v>
       </c>
       <c r="AD13" t="n">
-        <v>4.95</v>
+        <v>4.23</v>
       </c>
       <c r="AE13" t="n">
-        <v>408</v>
+        <v>981</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>44532</v>
+      <c r="A14" s="2" t="n">
+        <v>44623</v>
       </c>
       <c r="B14" t="n">
-        <v>44.21</v>
+        <v>37.67</v>
       </c>
       <c r="C14" t="n">
-        <v>18.71</v>
+        <v>12.35</v>
       </c>
       <c r="D14" t="n">
-        <v>5.35</v>
+        <v>8.1</v>
       </c>
       <c r="E14" t="n">
-        <v>4302</v>
+        <v>4288</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>29.06</v>
       </c>
       <c r="G14" t="n">
-        <v>2.22</v>
+        <v>1.78</v>
       </c>
       <c r="H14" t="n">
-        <v>101952090</v>
+        <v>85245420.00000001</v>
       </c>
       <c r="I14" t="n">
-        <v>7545</v>
+        <v>7611</v>
       </c>
       <c r="J14" t="n">
-        <v>9580</v>
+        <v>10122</v>
       </c>
       <c r="K14" t="n">
-        <v>-2035</v>
+        <v>-2511</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="N14" t="n">
-        <v>8.51</v>
+        <v>6.2</v>
       </c>
       <c r="O14" t="n">
-        <v>11.87</v>
+        <v>14.44</v>
       </c>
       <c r="P14" t="n">
-        <v>11.86</v>
+        <v>14.83</v>
       </c>
       <c r="Q14" t="n">
-        <v>3938</v>
+        <v>3628</v>
       </c>
       <c r="R14" t="n">
-        <v>-2485</v>
+        <v>-2691</v>
       </c>
       <c r="S14" t="n">
-        <v>-513</v>
+        <v>-466</v>
       </c>
       <c r="T14" t="n">
-        <v>673</v>
+        <v>1017</v>
       </c>
       <c r="U14" t="n">
-        <v>3265</v>
+        <v>2611</v>
       </c>
       <c r="V14" t="n">
-        <v>5016</v>
+        <v>4634</v>
       </c>
       <c r="W14" t="n">
-        <v>712</v>
+        <v>792</v>
       </c>
       <c r="X14" t="n">
-        <v>7686</v>
+        <v>7449</v>
       </c>
       <c r="Y14" t="n">
-        <v>13679</v>
+        <v>14584</v>
       </c>
       <c r="Z14" t="n">
-        <v>126.22</v>
+        <v>96.85000000000001</v>
       </c>
       <c r="AA14" t="n">
-        <v>7</v>
+        <v>1702</v>
       </c>
       <c r="AB14" t="n">
-        <v>624</v>
+        <v>2487</v>
       </c>
       <c r="AC14" t="n">
         <v>0.1</v>
       </c>
       <c r="AD14" t="n">
-        <v>4.86</v>
+        <v>4.95</v>
       </c>
       <c r="AE14" t="n">
-        <v>259</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>44350</v>
+      <c r="A15" s="2" t="n">
+        <v>44532</v>
       </c>
       <c r="B15" t="n">
-        <v>53.57</v>
+        <v>44.21</v>
       </c>
       <c r="C15" t="n">
-        <v>23.49</v>
+        <v>18.71</v>
       </c>
       <c r="D15" t="n">
-        <v>4.26</v>
+        <v>5.35</v>
       </c>
       <c r="E15" t="n">
-        <v>3356</v>
+        <v>4302</v>
       </c>
       <c r="F15" t="n">
-        <v>23.38</v>
+        <v>30</v>
       </c>
       <c r="G15" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="H15" t="n">
-        <v>92942110</v>
+        <v>101952090</v>
       </c>
       <c r="I15" t="n">
-        <v>7228</v>
+        <v>7545</v>
       </c>
       <c r="J15" t="n">
-        <v>8349</v>
+        <v>9580</v>
       </c>
       <c r="K15" t="n">
-        <v>-1121</v>
+        <v>-2035</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.11</v>
+        <v>-0.17</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="N15" t="n">
-        <v>9.19</v>
+        <v>8.51</v>
       </c>
       <c r="O15" t="n">
-        <v>9.33</v>
+        <v>11.87</v>
       </c>
       <c r="P15" t="n">
-        <v>8.99</v>
+        <v>11.86</v>
       </c>
       <c r="Q15" t="n">
-        <v>3560</v>
+        <v>3938</v>
       </c>
       <c r="R15" t="n">
-        <v>-2081</v>
+        <v>-2485</v>
       </c>
       <c r="S15" t="n">
-        <v>-228</v>
+        <v>-513</v>
       </c>
       <c r="T15" t="n">
-        <v>1301</v>
+        <v>673</v>
       </c>
       <c r="U15" t="n">
-        <v>2259</v>
+        <v>3265</v>
       </c>
       <c r="V15" t="n">
-        <v>3944</v>
+        <v>5016</v>
       </c>
       <c r="W15" t="n">
-        <v>670</v>
+        <v>712</v>
       </c>
       <c r="X15" t="n">
-        <v>6551</v>
+        <v>7686</v>
       </c>
       <c r="Y15" t="n">
-        <v>13099</v>
+        <v>13679</v>
       </c>
       <c r="Z15" t="n">
-        <v>152.23</v>
+        <v>126.22</v>
       </c>
       <c r="AA15" t="n">
-        <v>764</v>
+        <v>7</v>
       </c>
       <c r="AB15" t="n">
-        <v>52</v>
+        <v>624</v>
       </c>
       <c r="AC15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>4.86</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>44259</v>
+      <c r="A16" s="2" t="n">
+        <v>44350</v>
       </c>
       <c r="B16" t="n">
-        <v>159.86</v>
+        <v>53.57</v>
       </c>
       <c r="C16" t="n">
-        <v>36.78</v>
+        <v>23.49</v>
       </c>
       <c r="D16" t="n">
-        <v>2.72</v>
+        <v>4.26</v>
       </c>
       <c r="E16" t="n">
-        <v>2212</v>
+        <v>3356</v>
       </c>
       <c r="F16" t="n">
-        <v>9.67</v>
+        <v>23.38</v>
       </c>
       <c r="G16" t="n">
-        <v>2.37</v>
+        <v>2.2</v>
       </c>
       <c r="H16" t="n">
-        <v>96398400</v>
+        <v>92942110</v>
       </c>
       <c r="I16" t="n">
-        <v>7149</v>
+        <v>7228</v>
       </c>
       <c r="J16" t="n">
-        <v>7184</v>
+        <v>8349</v>
       </c>
       <c r="K16" t="n">
-        <v>-35</v>
+        <v>-1121</v>
       </c>
       <c r="L16" t="n">
-        <v>-0</v>
+        <v>-0.11</v>
       </c>
       <c r="M16" t="n">
-        <v>-0</v>
+        <v>-0.03</v>
       </c>
       <c r="N16" t="n">
-        <v>11.11</v>
+        <v>9.19</v>
       </c>
       <c r="O16" t="n">
-        <v>6.43</v>
+        <v>9.33</v>
       </c>
       <c r="P16" t="n">
-        <v>6.37</v>
+        <v>8.99</v>
       </c>
       <c r="Q16" t="n">
-        <v>3057</v>
+        <v>3560</v>
       </c>
       <c r="R16" t="n">
-        <v>-2556</v>
+        <v>-2081</v>
       </c>
       <c r="S16" t="n">
-        <v>5</v>
+        <v>-228</v>
       </c>
       <c r="T16" t="n">
-        <v>39</v>
+        <v>1301</v>
       </c>
       <c r="U16" t="n">
-        <v>3018</v>
+        <v>2259</v>
       </c>
       <c r="V16" t="n">
-        <v>3933</v>
+        <v>3944</v>
       </c>
       <c r="W16" t="n">
-        <v>641</v>
+        <v>670</v>
       </c>
       <c r="X16" t="n">
         <v>6551</v>
       </c>
       <c r="Y16" t="n">
-        <v>11846</v>
+        <v>13099</v>
       </c>
       <c r="Z16" t="n">
-        <v>188.83</v>
+        <v>152.23</v>
       </c>
       <c r="AA16" t="n">
-        <v>258</v>
+        <v>764</v>
       </c>
       <c r="AB16" t="n">
-        <v>-275</v>
+        <v>52</v>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
@@ -3002,97 +3034,192 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
+        <v>44259</v>
+      </c>
+      <c r="B17" t="n">
+        <v>159.86</v>
+      </c>
+      <c r="C17" t="n">
+        <v>36.78</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2212</v>
+      </c>
+      <c r="F17" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H17" t="n">
+        <v>96398400</v>
+      </c>
+      <c r="I17" t="n">
+        <v>7149</v>
+      </c>
+      <c r="J17" t="n">
+        <v>7184</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-35</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="O17" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3057</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-2556</v>
+      </c>
+      <c r="S17" t="n">
+        <v>5</v>
+      </c>
+      <c r="T17" t="n">
+        <v>39</v>
+      </c>
+      <c r="U17" t="n">
+        <v>3018</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3933</v>
+      </c>
+      <c r="W17" t="n">
+        <v>641</v>
+      </c>
+      <c r="X17" t="n">
+        <v>6551</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>11846</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>188.83</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>258</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>-275</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44168</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" t="n">
         <v>101.85</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>32.75</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>3.05</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>2353</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>13.91</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>2.05</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>81785250</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I18" t="n">
         <v>7158</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>7032</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>126</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>0.02</v>
       </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="n">
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O18" t="n">
         <v>6.27</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>6.18</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>1967</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-3418</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-214</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>-771</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>2738</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>3111</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>647</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>5728</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>10841</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>211.35</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>-395</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>-815</v>
       </c>
-      <c r="AC17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizacao dos dados do 3Q26 da MU
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/micron/mu_indicators.xlsx
+++ b/analise_eua/semicondutores/micron/mu_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>21.85</v>
+        <v>21.84</v>
       </c>
       <c r="C2" t="n">
-        <v>21.85</v>
+        <v>21.84</v>
       </c>
       <c r="D2" t="n">
         <v>4.58</v>
@@ -610,7 +610,7 @@
         <v>3.44</v>
       </c>
       <c r="H2" t="n">
-        <v>186539400</v>
+        <v>186461280</v>
       </c>
       <c r="I2" t="n">
         <v>15278</v>
@@ -628,7 +628,7 @@
         <v>0.09</v>
       </c>
       <c r="N2" t="n">
-        <v>10.57</v>
+        <v>10.56</v>
       </c>
       <c r="O2" t="n">
         <v>15.76</v>
@@ -687,10 +687,10 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>146.46</v>
+        <v>146.41</v>
       </c>
       <c r="C3" t="n">
-        <v>147.31</v>
+        <v>147.26</v>
       </c>
       <c r="D3" t="n">
         <v>0.68</v>
@@ -705,7 +705,7 @@
         <v>2.52</v>
       </c>
       <c r="H3" t="n">
-        <v>113947600</v>
+        <v>113903400</v>
       </c>
       <c r="I3" t="n">
         <v>14007</v>
@@ -788,7 +788,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-7.93</v>
+        <v>-7.94</v>
       </c>
       <c r="E4" t="n">
         <v>2011</v>
@@ -800,7 +800,7 @@
         <v>1.67</v>
       </c>
       <c r="H4" t="n">
-        <v>73580760</v>
+        <v>73547970</v>
       </c>
       <c r="I4" t="n">
         <v>13933</v>
@@ -818,7 +818,7 @@
         <v>0.1</v>
       </c>
       <c r="N4" t="n">
-        <v>38.75</v>
+        <v>38.73</v>
       </c>
       <c r="O4" t="n">
         <v>-13.22</v>
@@ -880,10 +880,10 @@
         <v>6.29</v>
       </c>
       <c r="C5" t="n">
-        <v>6.3</v>
+        <v>6.29</v>
       </c>
       <c r="D5" t="n">
-        <v>15.88</v>
+        <v>15.89</v>
       </c>
       <c r="E5" t="n">
         <v>16818</v>
@@ -895,7 +895,7 @@
         <v>1.1</v>
       </c>
       <c r="H5" t="n">
-        <v>54677040</v>
+        <v>54654799.99999999</v>
       </c>
       <c r="I5" t="n">
         <v>7516</v>
@@ -975,7 +975,7 @@
         <v>13.25</v>
       </c>
       <c r="C6" t="n">
-        <v>13.26</v>
+        <v>13.25</v>
       </c>
       <c r="D6" t="n">
         <v>7.54</v>
@@ -990,7 +990,7 @@
         <v>1.77</v>
       </c>
       <c r="H6" t="n">
-        <v>77672000</v>
+        <v>77638400</v>
       </c>
       <c r="I6" t="n">
         <v>7280</v>
@@ -1067,7 +1067,7 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>18.93</v>
+        <v>18.92</v>
       </c>
       <c r="C7" t="n">
         <v>18.93</v>
@@ -1085,7 +1085,7 @@
         <v>1.3</v>
       </c>
       <c r="H7" t="n">
-        <v>50860200</v>
+        <v>50838000</v>
       </c>
       <c r="I7" t="n">
         <v>7176</v>
@@ -1162,13 +1162,13 @@
         <v>2019</v>
       </c>
       <c r="B8" t="n">
-        <v>7.38</v>
+        <v>7.37</v>
       </c>
       <c r="C8" t="n">
         <v>7.37</v>
       </c>
       <c r="D8" t="n">
-        <v>13.56</v>
+        <v>13.57</v>
       </c>
       <c r="E8" t="n">
         <v>12800</v>
@@ -1180,7 +1180,7 @@
         <v>1.3</v>
       </c>
       <c r="H8" t="n">
-        <v>46576340.00000001</v>
+        <v>46554060</v>
       </c>
       <c r="I8" t="n">
         <v>5851</v>
@@ -1257,13 +1257,13 @@
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>3.6</v>
+        <v>3.59</v>
       </c>
       <c r="C9" t="n">
-        <v>3.6</v>
+        <v>3.59</v>
       </c>
       <c r="D9" t="n">
-        <v>27.8</v>
+        <v>27.82</v>
       </c>
       <c r="E9" t="n">
         <v>19753</v>
@@ -1275,7 +1275,7 @@
         <v>1.57</v>
       </c>
       <c r="H9" t="n">
-        <v>50837760</v>
+        <v>50814720</v>
       </c>
       <c r="I9" t="n">
         <v>4636</v>
@@ -1355,7 +1355,7 @@
         <v>8.210000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>8.220000000000001</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="D10" t="n">
         <v>12.17</v>
@@ -1370,7 +1370,7 @@
         <v>2.24</v>
       </c>
       <c r="H10" t="n">
-        <v>41784930</v>
+        <v>41774040</v>
       </c>
       <c r="I10" t="n">
         <v>11134</v>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1610,379 +1610,379 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46107</v>
+        <v>46201</v>
       </c>
       <c r="B2" t="n">
-        <v>29.04</v>
+        <v>41.88</v>
       </c>
       <c r="C2" t="n">
-        <v>17.76</v>
+        <v>24.03</v>
       </c>
       <c r="D2" t="n">
-        <v>5.63</v>
+        <v>4.16</v>
       </c>
       <c r="E2" t="n">
-        <v>18421</v>
+        <v>35682</v>
       </c>
       <c r="F2" t="n">
-        <v>57.77</v>
+        <v>68.13</v>
       </c>
       <c r="G2" t="n">
-        <v>5.52</v>
+        <v>11.74</v>
       </c>
       <c r="H2" t="n">
-        <v>400247959.9999999</v>
+        <v>1182719280</v>
       </c>
       <c r="I2" t="n">
-        <v>10798</v>
+        <v>6376</v>
       </c>
       <c r="J2" t="n">
-        <v>14589</v>
+        <v>26022</v>
       </c>
       <c r="K2" t="n">
-        <v>-3791</v>
+        <v>-19646</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.11</v>
+        <v>-0.29</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="N2" t="n">
-        <v>11.58</v>
+        <v>18.02</v>
       </c>
       <c r="O2" t="n">
-        <v>31.04</v>
+        <v>48.8</v>
       </c>
       <c r="P2" t="n">
-        <v>35.82</v>
+        <v>61.78</v>
       </c>
       <c r="Q2" t="n">
-        <v>11903</v>
+        <v>25388</v>
       </c>
       <c r="R2" t="n">
-        <v>-5525</v>
+        <v>-9569</v>
       </c>
       <c r="S2" t="n">
-        <v>-2167</v>
+        <v>-4734</v>
       </c>
       <c r="T2" t="n">
-        <v>5516</v>
+        <v>17562</v>
       </c>
       <c r="U2" t="n">
-        <v>6387</v>
+        <v>7826</v>
       </c>
       <c r="V2" t="n">
-        <v>10098</v>
+        <v>13584</v>
       </c>
       <c r="W2" t="n">
-        <v>1250</v>
+        <v>1316</v>
       </c>
       <c r="X2" t="n">
-        <v>14382</v>
+        <v>18286</v>
       </c>
       <c r="Y2" t="n">
-        <v>27117</v>
+        <v>47249</v>
       </c>
       <c r="Z2" t="n">
-        <v>67.32000000000001</v>
+        <v>41.06</v>
       </c>
       <c r="AA2" t="n">
-        <v>2982</v>
+        <v>18075</v>
       </c>
       <c r="AB2" t="n">
-        <v>10418</v>
+        <v>35290</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.96</v>
+        <v>0.61</v>
       </c>
       <c r="AE2" t="n">
-        <v>350</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46018</v>
+        <v>46107</v>
       </c>
       <c r="B3" t="n">
-        <v>61.28</v>
+        <v>27.6</v>
       </c>
       <c r="C3" t="n">
-        <v>30.2</v>
+        <v>16.88</v>
       </c>
       <c r="D3" t="n">
-        <v>3.31</v>
+        <v>5.92</v>
       </c>
       <c r="E3" t="n">
-        <v>8348</v>
+        <v>18421</v>
       </c>
       <c r="F3" t="n">
-        <v>38.41</v>
+        <v>57.77</v>
       </c>
       <c r="G3" t="n">
-        <v>5.46</v>
+        <v>5.25</v>
       </c>
       <c r="H3" t="n">
-        <v>321086250</v>
+        <v>380407839.9999999</v>
       </c>
       <c r="I3" t="n">
-        <v>12425</v>
+        <v>10798</v>
       </c>
       <c r="J3" t="n">
-        <v>10318</v>
+        <v>14589</v>
       </c>
       <c r="K3" t="n">
-        <v>2107</v>
+        <v>-3791</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="N3" t="n">
-        <v>15.64</v>
+        <v>11.01</v>
       </c>
       <c r="O3" t="n">
-        <v>17.99</v>
+        <v>31.04</v>
       </c>
       <c r="P3" t="n">
-        <v>19.34</v>
+        <v>35.82</v>
       </c>
       <c r="Q3" t="n">
-        <v>8411</v>
+        <v>11903</v>
       </c>
       <c r="R3" t="n">
-        <v>-4594</v>
+        <v>-5525</v>
       </c>
       <c r="S3" t="n">
-        <v>-3745</v>
+        <v>-2167</v>
       </c>
       <c r="T3" t="n">
-        <v>3022</v>
+        <v>5516</v>
       </c>
       <c r="U3" t="n">
-        <v>5389</v>
+        <v>6387</v>
       </c>
       <c r="V3" t="n">
-        <v>7173</v>
+        <v>10098</v>
       </c>
       <c r="W3" t="n">
-        <v>1171</v>
+        <v>1250</v>
       </c>
       <c r="X3" t="n">
-        <v>11095</v>
+        <v>14382</v>
       </c>
       <c r="Y3" t="n">
-        <v>17605</v>
+        <v>27117</v>
       </c>
       <c r="Z3" t="n">
-        <v>81.38</v>
+        <v>67.32000000000001</v>
       </c>
       <c r="AA3" t="n">
-        <v>1172</v>
+        <v>2982</v>
       </c>
       <c r="AB3" t="n">
-        <v>4963</v>
+        <v>10418</v>
       </c>
       <c r="AC3" t="n">
         <v>0.12</v>
       </c>
       <c r="AD3" t="n">
-        <v>2.56</v>
+        <v>0.96</v>
       </c>
       <c r="AE3" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45837</v>
+        <v>46018</v>
       </c>
       <c r="B4" t="n">
-        <v>72.95999999999999</v>
+        <v>61.25</v>
       </c>
       <c r="C4" t="n">
-        <v>24.17</v>
+        <v>30.19</v>
       </c>
       <c r="D4" t="n">
-        <v>4.14</v>
+        <v>3.31</v>
       </c>
       <c r="E4" t="n">
-        <v>4263</v>
+        <v>8348</v>
       </c>
       <c r="F4" t="n">
-        <v>20.27</v>
+        <v>38.41</v>
       </c>
       <c r="G4" t="n">
-        <v>2.71</v>
+        <v>5.46</v>
       </c>
       <c r="H4" t="n">
-        <v>137525180</v>
+        <v>320951250</v>
       </c>
       <c r="I4" t="n">
-        <v>16141</v>
+        <v>12425</v>
       </c>
       <c r="J4" t="n">
-        <v>10811</v>
+        <v>10318</v>
       </c>
       <c r="K4" t="n">
-        <v>5330</v>
+        <v>2107</v>
       </c>
       <c r="L4" t="n">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="M4" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="N4" t="n">
-        <v>9.529999999999999</v>
+        <v>15.63</v>
       </c>
       <c r="O4" t="n">
-        <v>11.17</v>
+        <v>17.99</v>
       </c>
       <c r="P4" t="n">
-        <v>11.82</v>
+        <v>19.34</v>
       </c>
       <c r="Q4" t="n">
-        <v>4609</v>
+        <v>8411</v>
       </c>
       <c r="R4" t="n">
-        <v>-2589</v>
+        <v>-4594</v>
       </c>
       <c r="S4" t="n">
-        <v>540</v>
+        <v>-3745</v>
       </c>
       <c r="T4" t="n">
-        <v>1671</v>
+        <v>3022</v>
       </c>
       <c r="U4" t="n">
-        <v>2938</v>
+        <v>5389</v>
       </c>
       <c r="V4" t="n">
-        <v>4127</v>
+        <v>7173</v>
       </c>
       <c r="W4" t="n">
-        <v>965</v>
+        <v>1171</v>
       </c>
       <c r="X4" t="n">
-        <v>7728</v>
+        <v>11095</v>
       </c>
       <c r="Y4" t="n">
-        <v>17784</v>
+        <v>17605</v>
       </c>
       <c r="Z4" t="n">
-        <v>95.09</v>
+        <v>81.38</v>
       </c>
       <c r="AA4" t="n">
-        <v>1863</v>
+        <v>1172</v>
       </c>
       <c r="AB4" t="n">
-        <v>2917</v>
+        <v>4963</v>
       </c>
       <c r="AC4" t="n">
         <v>0.12</v>
       </c>
       <c r="AD4" t="n">
-        <v>6.95</v>
+        <v>2.56</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45743</v>
+        <v>45837</v>
       </c>
       <c r="B5" t="n">
-        <v>61.08</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>21.05</v>
+        <v>24.16</v>
       </c>
       <c r="D5" t="n">
-        <v>4.75</v>
+        <v>4.14</v>
       </c>
       <c r="E5" t="n">
-        <v>3852</v>
+        <v>4263</v>
       </c>
       <c r="F5" t="n">
-        <v>19.66</v>
+        <v>20.27</v>
       </c>
       <c r="G5" t="n">
-        <v>1.99</v>
+        <v>2.71</v>
       </c>
       <c r="H5" t="n">
-        <v>96692800</v>
+        <v>137469280</v>
       </c>
       <c r="I5" t="n">
-        <v>14954</v>
+        <v>16141</v>
       </c>
       <c r="J5" t="n">
-        <v>8215</v>
+        <v>10811</v>
       </c>
       <c r="K5" t="n">
-        <v>6739</v>
+        <v>5330</v>
       </c>
       <c r="L5" t="n">
-        <v>0.52</v>
+        <v>0.36</v>
       </c>
       <c r="M5" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="N5" t="n">
-        <v>8.050000000000001</v>
+        <v>9.52</v>
       </c>
       <c r="O5" t="n">
-        <v>9.41</v>
+        <v>11.17</v>
       </c>
       <c r="P5" t="n">
-        <v>7.98</v>
+        <v>11.82</v>
       </c>
       <c r="Q5" t="n">
-        <v>3942</v>
+        <v>4609</v>
       </c>
       <c r="R5" t="n">
-        <v>-3152</v>
+        <v>-2589</v>
       </c>
       <c r="S5" t="n">
-        <v>96</v>
+        <v>540</v>
       </c>
       <c r="T5" t="n">
-        <v>-113</v>
+        <v>1671</v>
       </c>
       <c r="U5" t="n">
-        <v>4055</v>
+        <v>2938</v>
       </c>
       <c r="V5" t="n">
-        <v>2743</v>
+        <v>4127</v>
       </c>
       <c r="W5" t="n">
-        <v>898</v>
+        <v>965</v>
       </c>
       <c r="X5" t="n">
-        <v>6211</v>
+        <v>7728</v>
       </c>
       <c r="Y5" t="n">
-        <v>16812</v>
+        <v>17784</v>
       </c>
       <c r="Z5" t="n">
-        <v>122.14</v>
+        <v>95.09</v>
       </c>
       <c r="AA5" t="n">
-        <v>1143</v>
+        <v>1863</v>
       </c>
       <c r="AB5" t="n">
-        <v>2130</v>
+        <v>2917</v>
       </c>
       <c r="AC5" t="n">
         <v>0.12</v>
       </c>
       <c r="AD5" t="n">
-        <v>8.210000000000001</v>
+        <v>6.95</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1990,94 +1990,94 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45654</v>
+        <v>45743</v>
       </c>
       <c r="B6" t="n">
-        <v>49.84</v>
+        <v>61.05</v>
       </c>
       <c r="C6" t="n">
-        <v>53.09</v>
+        <v>21.04</v>
       </c>
       <c r="D6" t="n">
-        <v>1.88</v>
+        <v>4.75</v>
       </c>
       <c r="E6" t="n">
-        <v>4204</v>
+        <v>3852</v>
       </c>
       <c r="F6" t="n">
-        <v>21.47</v>
+        <v>19.66</v>
       </c>
       <c r="G6" t="n">
         <v>1.99</v>
       </c>
       <c r="H6" t="n">
-        <v>93201790</v>
+        <v>96648200.00000001</v>
       </c>
       <c r="I6" t="n">
-        <v>14373</v>
+        <v>14954</v>
       </c>
       <c r="J6" t="n">
-        <v>7588</v>
+        <v>8215</v>
       </c>
       <c r="K6" t="n">
-        <v>6785</v>
+        <v>6739</v>
       </c>
       <c r="L6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="M6" t="n">
         <v>0.14</v>
       </c>
       <c r="N6" t="n">
-        <v>10.22</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>3.76</v>
+        <v>9.41</v>
       </c>
       <c r="P6" t="n">
-        <v>3.38</v>
+        <v>7.98</v>
       </c>
       <c r="Q6" t="n">
-        <v>3244</v>
+        <v>3942</v>
       </c>
       <c r="R6" t="n">
-        <v>-3148</v>
+        <v>-3152</v>
       </c>
       <c r="S6" t="n">
-        <v>-422</v>
+        <v>96</v>
       </c>
       <c r="T6" t="n">
-        <v>38</v>
+        <v>-113</v>
       </c>
       <c r="U6" t="n">
-        <v>3206</v>
+        <v>4055</v>
       </c>
       <c r="V6" t="n">
-        <v>648</v>
+        <v>2743</v>
       </c>
       <c r="W6" t="n">
-        <v>888</v>
+        <v>898</v>
       </c>
       <c r="X6" t="n">
-        <v>4063</v>
+        <v>6211</v>
       </c>
       <c r="Y6" t="n">
-        <v>15478</v>
+        <v>16812</v>
       </c>
       <c r="Z6" t="n">
-        <v>247.31</v>
+        <v>122.14</v>
       </c>
       <c r="AA6" t="n">
-        <v>-837</v>
+        <v>1143</v>
       </c>
       <c r="AB6" t="n">
-        <v>259</v>
+        <v>2130</v>
       </c>
       <c r="AC6" t="n">
         <v>0.12</v>
       </c>
       <c r="AD6" t="n">
-        <v>7.01</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -2085,94 +2085,94 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45654</v>
       </c>
       <c r="B7" t="n">
-        <v>435.7</v>
+        <v>49.82</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>53.07</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.4</v>
+        <v>1.88</v>
       </c>
       <c r="E7" t="n">
-        <v>2674</v>
+        <v>4204</v>
       </c>
       <c r="F7" t="n">
-        <v>4.87</v>
+        <v>21.47</v>
       </c>
       <c r="G7" t="n">
-        <v>3.27</v>
+        <v>1.99</v>
       </c>
       <c r="H7" t="n">
-        <v>144651690</v>
+        <v>93157349.99999999</v>
       </c>
       <c r="I7" t="n">
-        <v>13867</v>
+        <v>14373</v>
       </c>
       <c r="J7" t="n">
-        <v>8379</v>
+        <v>7588</v>
       </c>
       <c r="K7" t="n">
-        <v>5488</v>
+        <v>6785</v>
       </c>
       <c r="L7" t="n">
-        <v>0.95</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="N7" t="n">
-        <v>26.02</v>
+        <v>10.22</v>
       </c>
       <c r="O7" t="n">
-        <v>-4.53</v>
+        <v>3.76</v>
       </c>
       <c r="P7" t="n">
-        <v>-3.46</v>
+        <v>3.38</v>
       </c>
       <c r="Q7" t="n">
-        <v>2482</v>
+        <v>3244</v>
       </c>
       <c r="R7" t="n">
-        <v>-2002</v>
+        <v>-3148</v>
       </c>
       <c r="S7" t="n">
-        <v>-910</v>
+        <v>-422</v>
       </c>
       <c r="T7" t="n">
-        <v>396</v>
+        <v>38</v>
       </c>
       <c r="U7" t="n">
-        <v>2086</v>
+        <v>3206</v>
       </c>
       <c r="V7" t="n">
-        <v>-923</v>
+        <v>648</v>
       </c>
       <c r="W7" t="n">
-        <v>850</v>
+        <v>888</v>
       </c>
       <c r="X7" t="n">
-        <v>2362</v>
+        <v>4063</v>
       </c>
       <c r="Y7" t="n">
-        <v>16479</v>
+        <v>15478</v>
       </c>
       <c r="Z7" t="n">
-        <v>-125.89</v>
+        <v>247.31</v>
       </c>
       <c r="AA7" t="n">
-        <v>-1228</v>
+        <v>-837</v>
       </c>
       <c r="AB7" t="n">
-        <v>-2270</v>
+        <v>259</v>
       </c>
       <c r="AC7" t="n">
         <v>0.12</v>
       </c>
       <c r="AD7" t="n">
-        <v>38.55</v>
+        <v>7.01</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -2180,94 +2180,94 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45380</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>163.05</v>
+        <v>435.5</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>-3.63</v>
+        <v>-1.4</v>
       </c>
       <c r="E8" t="n">
-        <v>2115</v>
+        <v>2674</v>
       </c>
       <c r="F8" t="n">
-        <v>13.62</v>
+        <v>4.87</v>
       </c>
       <c r="G8" t="n">
-        <v>2.95</v>
+        <v>3.27</v>
       </c>
       <c r="H8" t="n">
-        <v>129300480</v>
+        <v>144585270</v>
       </c>
       <c r="I8" t="n">
-        <v>14315</v>
+        <v>13867</v>
       </c>
       <c r="J8" t="n">
-        <v>9006</v>
+        <v>8379</v>
       </c>
       <c r="K8" t="n">
-        <v>5309</v>
+        <v>5488</v>
       </c>
       <c r="L8" t="n">
-        <v>1.94</v>
+        <v>0.95</v>
       </c>
       <c r="M8" t="n">
         <v>0.12</v>
       </c>
       <c r="N8" t="n">
-        <v>49.2</v>
+        <v>26</v>
       </c>
       <c r="O8" t="n">
-        <v>-10.6</v>
+        <v>-4.53</v>
       </c>
       <c r="P8" t="n">
-        <v>-9.210000000000001</v>
+        <v>-3.46</v>
       </c>
       <c r="Q8" t="n">
-        <v>1219</v>
+        <v>2482</v>
       </c>
       <c r="R8" t="n">
-        <v>-1151</v>
+        <v>-2002</v>
       </c>
       <c r="S8" t="n">
-        <v>-106</v>
+        <v>-910</v>
       </c>
       <c r="T8" t="n">
-        <v>-165</v>
+        <v>396</v>
       </c>
       <c r="U8" t="n">
-        <v>1384</v>
+        <v>2086</v>
       </c>
       <c r="V8" t="n">
-        <v>-791</v>
+        <v>-923</v>
       </c>
       <c r="W8" t="n">
-        <v>832</v>
+        <v>850</v>
       </c>
       <c r="X8" t="n">
-        <v>2432</v>
+        <v>2362</v>
       </c>
       <c r="Y8" t="n">
-        <v>17176</v>
+        <v>16479</v>
       </c>
       <c r="Z8" t="n">
-        <v>-78.92</v>
+        <v>-125.89</v>
       </c>
       <c r="AA8" t="n">
-        <v>-3075</v>
+        <v>-1228</v>
       </c>
       <c r="AB8" t="n">
-        <v>-6006</v>
+        <v>-2270</v>
       </c>
       <c r="AC8" t="n">
         <v>0.12</v>
       </c>
       <c r="AD8" t="n">
-        <v>16.02</v>
+        <v>38.55</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -2275,94 +2275,94 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45290</v>
+        <v>45380</v>
       </c>
       <c r="B9" t="n">
-        <v>-75.5</v>
+        <v>162.98</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-6.08</v>
+        <v>-3.63</v>
       </c>
       <c r="E9" t="n">
-        <v>787</v>
+        <v>2115</v>
       </c>
       <c r="F9" t="n">
-        <v>-26.11</v>
+        <v>13.62</v>
       </c>
       <c r="G9" t="n">
-        <v>2.17</v>
+        <v>2.95</v>
       </c>
       <c r="H9" t="n">
-        <v>93170000</v>
+        <v>129245280</v>
       </c>
       <c r="I9" t="n">
-        <v>14106</v>
+        <v>14315</v>
       </c>
       <c r="J9" t="n">
-        <v>9048</v>
+        <v>9006</v>
       </c>
       <c r="K9" t="n">
-        <v>5058</v>
+        <v>5309</v>
       </c>
       <c r="L9" t="n">
-        <v>2.17</v>
+        <v>1.94</v>
       </c>
       <c r="M9" t="n">
         <v>0.12</v>
       </c>
       <c r="N9" t="n">
-        <v>42.1</v>
+        <v>49.18</v>
       </c>
       <c r="O9" t="n">
-        <v>-13.14</v>
+        <v>-10.6</v>
       </c>
       <c r="P9" t="n">
-        <v>-9</v>
+        <v>-9.210000000000001</v>
       </c>
       <c r="Q9" t="n">
-        <v>1401</v>
+        <v>1219</v>
       </c>
       <c r="R9" t="n">
-        <v>-1558</v>
+        <v>-1151</v>
       </c>
       <c r="S9" t="n">
-        <v>-352</v>
+        <v>-106</v>
       </c>
       <c r="T9" t="n">
-        <v>-395</v>
+        <v>-165</v>
       </c>
       <c r="U9" t="n">
-        <v>1796</v>
+        <v>1384</v>
       </c>
       <c r="V9" t="n">
-        <v>277</v>
+        <v>-791</v>
       </c>
       <c r="W9" t="n">
-        <v>845</v>
+        <v>832</v>
       </c>
       <c r="X9" t="n">
-        <v>3517</v>
+        <v>2432</v>
       </c>
       <c r="Y9" t="n">
-        <v>15096</v>
+        <v>17176</v>
       </c>
       <c r="Z9" t="n">
-        <v>-59.63</v>
+        <v>-78.92</v>
       </c>
       <c r="AA9" t="n">
-        <v>503</v>
+        <v>-3075</v>
       </c>
       <c r="AB9" t="n">
-        <v>-5218</v>
+        <v>-6006</v>
       </c>
       <c r="AC9" t="n">
         <v>0.12</v>
       </c>
       <c r="AD9" t="n">
-        <v>-10.45</v>
+        <v>16.02</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2370,94 +2370,94 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45078</v>
+        <v>45290</v>
       </c>
       <c r="B10" t="n">
-        <v>-35.96</v>
+        <v>-75.47</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>-2.68</v>
+        <v>-6.08</v>
       </c>
       <c r="E10" t="n">
-        <v>195</v>
+        <v>787</v>
       </c>
       <c r="F10" t="n">
-        <v>-50.53</v>
+        <v>-26.11</v>
       </c>
       <c r="G10" t="n">
-        <v>1.5</v>
+        <v>2.17</v>
       </c>
       <c r="H10" t="n">
-        <v>68189020</v>
+        <v>93126000</v>
       </c>
       <c r="I10" t="n">
-        <v>13848</v>
+        <v>14106</v>
       </c>
       <c r="J10" t="n">
-        <v>10352</v>
+        <v>9048</v>
       </c>
       <c r="K10" t="n">
-        <v>3496</v>
+        <v>5058</v>
       </c>
       <c r="L10" t="n">
-        <v>0.55</v>
+        <v>2.17</v>
       </c>
       <c r="M10" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="N10" t="n">
-        <v>11.25</v>
+        <v>42.08</v>
       </c>
       <c r="O10" t="n">
-        <v>-3.91</v>
+        <v>-13.14</v>
       </c>
       <c r="P10" t="n">
-        <v>-1.2</v>
+        <v>-9</v>
       </c>
       <c r="Q10" t="n">
-        <v>24</v>
+        <v>1401</v>
       </c>
       <c r="R10" t="n">
-        <v>-1180</v>
+        <v>-1558</v>
       </c>
       <c r="S10" t="n">
-        <v>661</v>
+        <v>-352</v>
       </c>
       <c r="T10" t="n">
-        <v>-1537</v>
+        <v>-395</v>
       </c>
       <c r="U10" t="n">
-        <v>1561</v>
+        <v>1796</v>
       </c>
       <c r="V10" t="n">
-        <v>1153</v>
+        <v>277</v>
       </c>
       <c r="W10" t="n">
-        <v>758</v>
+        <v>845</v>
       </c>
       <c r="X10" t="n">
-        <v>4321</v>
+        <v>3517</v>
       </c>
       <c r="Y10" t="n">
-        <v>16630</v>
+        <v>15096</v>
       </c>
       <c r="Z10" t="n">
-        <v>-701.6899999999999</v>
+        <v>-59.63</v>
       </c>
       <c r="AA10" t="n">
-        <v>2392</v>
+        <v>503</v>
       </c>
       <c r="AB10" t="n">
-        <v>-3083</v>
+        <v>-5218</v>
       </c>
       <c r="AC10" t="n">
         <v>0.12</v>
       </c>
       <c r="AD10" t="n">
-        <v>-6.65</v>
+        <v>-10.45</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2465,94 +2465,94 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>44987</v>
+        <v>45078</v>
       </c>
       <c r="B11" t="n">
-        <v>-28.07</v>
+        <v>-35.95</v>
       </c>
       <c r="C11" t="n">
-        <v>28.6</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>3.5</v>
+        <v>-2.68</v>
       </c>
       <c r="E11" t="n">
-        <v>-361</v>
+        <v>195</v>
       </c>
       <c r="F11" t="n">
-        <v>-62.6</v>
+        <v>-50.53</v>
       </c>
       <c r="G11" t="n">
-        <v>1.37</v>
+        <v>1.5</v>
       </c>
       <c r="H11" t="n">
-        <v>64892679.99999999</v>
+        <v>68156200</v>
       </c>
       <c r="I11" t="n">
-        <v>12884</v>
+        <v>13848</v>
       </c>
       <c r="J11" t="n">
-        <v>10818</v>
+        <v>10352</v>
       </c>
       <c r="K11" t="n">
-        <v>2066</v>
+        <v>3496</v>
       </c>
       <c r="L11" t="n">
-        <v>0.2</v>
+        <v>0.55</v>
       </c>
       <c r="M11" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="N11" t="n">
-        <v>6.4</v>
+        <v>11.25</v>
       </c>
       <c r="O11" t="n">
-        <v>5.04</v>
+        <v>-3.91</v>
       </c>
       <c r="P11" t="n">
-        <v>6.17</v>
+        <v>-1.2</v>
       </c>
       <c r="Q11" t="n">
-        <v>343</v>
+        <v>24</v>
       </c>
       <c r="R11" t="n">
-        <v>-1915</v>
+        <v>-1180</v>
       </c>
       <c r="S11" t="n">
-        <v>1802</v>
+        <v>661</v>
       </c>
       <c r="T11" t="n">
-        <v>-1862</v>
+        <v>-1537</v>
       </c>
       <c r="U11" t="n">
-        <v>2205</v>
+        <v>1561</v>
       </c>
       <c r="V11" t="n">
-        <v>2417</v>
+        <v>1153</v>
       </c>
       <c r="W11" t="n">
-        <v>788</v>
+        <v>758</v>
       </c>
       <c r="X11" t="n">
-        <v>5619</v>
+        <v>4321</v>
       </c>
       <c r="Y11" t="n">
-        <v>16643</v>
+        <v>16630</v>
       </c>
       <c r="Z11" t="n">
-        <v>174.76</v>
+        <v>-701.6899999999999</v>
       </c>
       <c r="AA11" t="n">
-        <v>4204</v>
+        <v>2392</v>
       </c>
       <c r="AB11" t="n">
-        <v>-321</v>
+        <v>-3083</v>
       </c>
       <c r="AC11" t="n">
         <v>0.12</v>
       </c>
       <c r="AD11" t="n">
-        <v>-5.45</v>
+        <v>-6.65</v>
       </c>
       <c r="AE11" t="n">
         <v>0</v>
@@ -2560,563 +2560,563 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44896</v>
+        <v>44987</v>
       </c>
       <c r="B12" t="n">
-        <v>-275.35</v>
+        <v>-28.05</v>
       </c>
       <c r="C12" t="n">
-        <v>7.87</v>
+        <v>28.58</v>
       </c>
       <c r="D12" t="n">
-        <v>12.71</v>
+        <v>3.5</v>
       </c>
       <c r="E12" t="n">
-        <v>1712</v>
+        <v>-361</v>
       </c>
       <c r="F12" t="n">
-        <v>-4.77</v>
+        <v>-62.6</v>
       </c>
       <c r="G12" t="n">
-        <v>1.09</v>
+        <v>1.37</v>
       </c>
       <c r="H12" t="n">
-        <v>53693400</v>
+        <v>64859950.00000001</v>
       </c>
       <c r="I12" t="n">
-        <v>10890</v>
+        <v>12884</v>
       </c>
       <c r="J12" t="n">
-        <v>10581</v>
+        <v>10818</v>
       </c>
       <c r="K12" t="n">
-        <v>309</v>
+        <v>2066</v>
       </c>
       <c r="L12" t="n">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="M12" t="n">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="N12" t="n">
-        <v>3.57</v>
+        <v>6.4</v>
       </c>
       <c r="O12" t="n">
-        <v>14.2</v>
+        <v>5.04</v>
       </c>
       <c r="P12" t="n">
-        <v>14.64</v>
+        <v>6.17</v>
       </c>
       <c r="Q12" t="n">
-        <v>943</v>
+        <v>343</v>
       </c>
       <c r="R12" t="n">
-        <v>-2266</v>
+        <v>-1915</v>
       </c>
       <c r="S12" t="n">
-        <v>2632</v>
+        <v>1802</v>
       </c>
       <c r="T12" t="n">
-        <v>-1506</v>
+        <v>-1862</v>
       </c>
       <c r="U12" t="n">
-        <v>2449</v>
+        <v>2205</v>
       </c>
       <c r="V12" t="n">
-        <v>3748</v>
+        <v>2417</v>
       </c>
       <c r="W12" t="n">
-        <v>849</v>
+        <v>788</v>
       </c>
       <c r="X12" t="n">
-        <v>6874</v>
+        <v>5619</v>
       </c>
       <c r="Y12" t="n">
-        <v>16396</v>
+        <v>16643</v>
       </c>
       <c r="Z12" t="n">
-        <v>88.34999999999999</v>
+        <v>174.76</v>
       </c>
       <c r="AA12" t="n">
-        <v>5662</v>
+        <v>4204</v>
       </c>
       <c r="AB12" t="n">
-        <v>2951</v>
+        <v>-321</v>
       </c>
       <c r="AC12" t="n">
         <v>0.12</v>
       </c>
       <c r="AD12" t="n">
-        <v>-64.62</v>
+        <v>-5.45</v>
       </c>
       <c r="AE12" t="n">
-        <v>425</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44714</v>
+        <v>44896</v>
       </c>
       <c r="B13" t="n">
-        <v>22.93</v>
+        <v>-275.24</v>
       </c>
       <c r="C13" t="n">
-        <v>6.78</v>
+        <v>7.87</v>
       </c>
       <c r="D13" t="n">
-        <v>14.76</v>
+        <v>12.71</v>
       </c>
       <c r="E13" t="n">
-        <v>4825</v>
+        <v>1712</v>
       </c>
       <c r="F13" t="n">
-        <v>30.39</v>
+        <v>-4.77</v>
       </c>
       <c r="G13" t="n">
-        <v>1.22</v>
+        <v>1.09</v>
       </c>
       <c r="H13" t="n">
-        <v>60203680</v>
+        <v>53671600</v>
       </c>
       <c r="I13" t="n">
-        <v>7592</v>
+        <v>10890</v>
       </c>
       <c r="J13" t="n">
-        <v>10227</v>
+        <v>10581</v>
       </c>
       <c r="K13" t="n">
-        <v>-2635</v>
+        <v>309</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.16</v>
+        <v>0.02</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.05</v>
+        <v>0.01</v>
       </c>
       <c r="N13" t="n">
-        <v>3.75</v>
+        <v>3.57</v>
       </c>
       <c r="O13" t="n">
-        <v>18.12</v>
+        <v>14.2</v>
       </c>
       <c r="P13" t="n">
-        <v>19.13</v>
+        <v>14.64</v>
       </c>
       <c r="Q13" t="n">
-        <v>3838</v>
+        <v>943</v>
       </c>
       <c r="R13" t="n">
-        <v>-2585</v>
+        <v>-2266</v>
       </c>
       <c r="S13" t="n">
-        <v>-1161</v>
+        <v>2632</v>
       </c>
       <c r="T13" t="n">
-        <v>1260</v>
+        <v>-1506</v>
       </c>
       <c r="U13" t="n">
-        <v>2578</v>
+        <v>2449</v>
       </c>
       <c r="V13" t="n">
-        <v>3922</v>
+        <v>3748</v>
       </c>
       <c r="W13" t="n">
-        <v>773</v>
+        <v>849</v>
       </c>
       <c r="X13" t="n">
-        <v>6869</v>
+        <v>6874</v>
       </c>
       <c r="Y13" t="n">
-        <v>15699</v>
+        <v>16396</v>
       </c>
       <c r="Z13" t="n">
-        <v>70.81</v>
+        <v>88.34999999999999</v>
       </c>
       <c r="AA13" t="n">
-        <v>4114</v>
+        <v>5662</v>
       </c>
       <c r="AB13" t="n">
-        <v>5225</v>
+        <v>2951</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="AD13" t="n">
-        <v>4.23</v>
+        <v>-64.62</v>
       </c>
       <c r="AE13" t="n">
-        <v>981</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44623</v>
+        <v>44714</v>
       </c>
       <c r="B14" t="n">
-        <v>37.67</v>
+        <v>22.92</v>
       </c>
       <c r="C14" t="n">
-        <v>12.35</v>
+        <v>6.77</v>
       </c>
       <c r="D14" t="n">
-        <v>8.1</v>
+        <v>14.76</v>
       </c>
       <c r="E14" t="n">
-        <v>4288</v>
+        <v>4825</v>
       </c>
       <c r="F14" t="n">
-        <v>29.06</v>
+        <v>30.39</v>
       </c>
       <c r="G14" t="n">
-        <v>1.78</v>
+        <v>1.22</v>
       </c>
       <c r="H14" t="n">
-        <v>85245420.00000001</v>
+        <v>60181439.99999999</v>
       </c>
       <c r="I14" t="n">
-        <v>7611</v>
+        <v>7592</v>
       </c>
       <c r="J14" t="n">
-        <v>10122</v>
+        <v>10227</v>
       </c>
       <c r="K14" t="n">
-        <v>-2511</v>
+        <v>-2635</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.18</v>
+        <v>-0.16</v>
       </c>
       <c r="M14" t="n">
         <v>-0.05</v>
       </c>
       <c r="N14" t="n">
-        <v>6.2</v>
+        <v>3.75</v>
       </c>
       <c r="O14" t="n">
-        <v>14.44</v>
+        <v>18.12</v>
       </c>
       <c r="P14" t="n">
-        <v>14.83</v>
+        <v>19.13</v>
       </c>
       <c r="Q14" t="n">
-        <v>3628</v>
+        <v>3838</v>
       </c>
       <c r="R14" t="n">
-        <v>-2691</v>
+        <v>-2585</v>
       </c>
       <c r="S14" t="n">
-        <v>-466</v>
+        <v>-1161</v>
       </c>
       <c r="T14" t="n">
-        <v>1017</v>
+        <v>1260</v>
       </c>
       <c r="U14" t="n">
-        <v>2611</v>
+        <v>2578</v>
       </c>
       <c r="V14" t="n">
-        <v>4634</v>
+        <v>3922</v>
       </c>
       <c r="W14" t="n">
-        <v>792</v>
+        <v>773</v>
       </c>
       <c r="X14" t="n">
-        <v>7449</v>
+        <v>6869</v>
       </c>
       <c r="Y14" t="n">
-        <v>14584</v>
+        <v>15699</v>
       </c>
       <c r="Z14" t="n">
-        <v>96.85000000000001</v>
+        <v>70.81</v>
       </c>
       <c r="AA14" t="n">
-        <v>1702</v>
+        <v>4114</v>
       </c>
       <c r="AB14" t="n">
-        <v>2487</v>
+        <v>5225</v>
       </c>
       <c r="AC14" t="n">
         <v>0.1</v>
       </c>
       <c r="AD14" t="n">
-        <v>4.95</v>
+        <v>4.23</v>
       </c>
       <c r="AE14" t="n">
-        <v>408</v>
+        <v>981</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44532</v>
+        <v>44623</v>
       </c>
       <c r="B15" t="n">
-        <v>44.21</v>
+        <v>37.65</v>
       </c>
       <c r="C15" t="n">
-        <v>18.71</v>
+        <v>12.34</v>
       </c>
       <c r="D15" t="n">
-        <v>5.35</v>
+        <v>8.1</v>
       </c>
       <c r="E15" t="n">
-        <v>4302</v>
+        <v>4288</v>
       </c>
       <c r="F15" t="n">
-        <v>30</v>
+        <v>29.06</v>
       </c>
       <c r="G15" t="n">
-        <v>2.22</v>
+        <v>1.78</v>
       </c>
       <c r="H15" t="n">
-        <v>101952090</v>
+        <v>85211850</v>
       </c>
       <c r="I15" t="n">
-        <v>7545</v>
+        <v>7611</v>
       </c>
       <c r="J15" t="n">
-        <v>9580</v>
+        <v>10122</v>
       </c>
       <c r="K15" t="n">
-        <v>-2035</v>
+        <v>-2511</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.04</v>
+        <v>-0.05</v>
       </c>
       <c r="N15" t="n">
-        <v>8.51</v>
+        <v>6.2</v>
       </c>
       <c r="O15" t="n">
-        <v>11.87</v>
+        <v>14.44</v>
       </c>
       <c r="P15" t="n">
-        <v>11.86</v>
+        <v>14.83</v>
       </c>
       <c r="Q15" t="n">
-        <v>3938</v>
+        <v>3628</v>
       </c>
       <c r="R15" t="n">
-        <v>-2485</v>
+        <v>-2691</v>
       </c>
       <c r="S15" t="n">
-        <v>-513</v>
+        <v>-466</v>
       </c>
       <c r="T15" t="n">
-        <v>673</v>
+        <v>1017</v>
       </c>
       <c r="U15" t="n">
-        <v>3265</v>
+        <v>2611</v>
       </c>
       <c r="V15" t="n">
-        <v>5016</v>
+        <v>4634</v>
       </c>
       <c r="W15" t="n">
-        <v>712</v>
+        <v>792</v>
       </c>
       <c r="X15" t="n">
-        <v>7686</v>
+        <v>7449</v>
       </c>
       <c r="Y15" t="n">
-        <v>13679</v>
+        <v>14584</v>
       </c>
       <c r="Z15" t="n">
-        <v>126.22</v>
+        <v>96.85000000000001</v>
       </c>
       <c r="AA15" t="n">
-        <v>7</v>
+        <v>1702</v>
       </c>
       <c r="AB15" t="n">
-        <v>624</v>
+        <v>2487</v>
       </c>
       <c r="AC15" t="n">
         <v>0.1</v>
       </c>
       <c r="AD15" t="n">
-        <v>4.86</v>
+        <v>4.95</v>
       </c>
       <c r="AE15" t="n">
-        <v>259</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44350</v>
+        <v>44532</v>
       </c>
       <c r="B16" t="n">
-        <v>53.57</v>
+        <v>44.19</v>
       </c>
       <c r="C16" t="n">
-        <v>23.49</v>
+        <v>18.7</v>
       </c>
       <c r="D16" t="n">
-        <v>4.26</v>
+        <v>5.35</v>
       </c>
       <c r="E16" t="n">
-        <v>3356</v>
+        <v>4302</v>
       </c>
       <c r="F16" t="n">
-        <v>23.38</v>
+        <v>30</v>
       </c>
       <c r="G16" t="n">
-        <v>2.2</v>
+        <v>2.22</v>
       </c>
       <c r="H16" t="n">
-        <v>92942110</v>
+        <v>101907330</v>
       </c>
       <c r="I16" t="n">
-        <v>7228</v>
+        <v>7545</v>
       </c>
       <c r="J16" t="n">
-        <v>8349</v>
+        <v>9580</v>
       </c>
       <c r="K16" t="n">
-        <v>-1121</v>
+        <v>-2035</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.11</v>
+        <v>-0.17</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="N16" t="n">
-        <v>9.19</v>
+        <v>8.5</v>
       </c>
       <c r="O16" t="n">
-        <v>9.33</v>
+        <v>11.87</v>
       </c>
       <c r="P16" t="n">
-        <v>8.99</v>
+        <v>11.86</v>
       </c>
       <c r="Q16" t="n">
-        <v>3560</v>
+        <v>3938</v>
       </c>
       <c r="R16" t="n">
-        <v>-2081</v>
+        <v>-2485</v>
       </c>
       <c r="S16" t="n">
-        <v>-228</v>
+        <v>-513</v>
       </c>
       <c r="T16" t="n">
-        <v>1301</v>
+        <v>673</v>
       </c>
       <c r="U16" t="n">
-        <v>2259</v>
+        <v>3265</v>
       </c>
       <c r="V16" t="n">
-        <v>3944</v>
+        <v>5016</v>
       </c>
       <c r="W16" t="n">
-        <v>670</v>
+        <v>712</v>
       </c>
       <c r="X16" t="n">
-        <v>6551</v>
+        <v>7686</v>
       </c>
       <c r="Y16" t="n">
-        <v>13099</v>
+        <v>13679</v>
       </c>
       <c r="Z16" t="n">
-        <v>152.23</v>
+        <v>126.22</v>
       </c>
       <c r="AA16" t="n">
-        <v>764</v>
+        <v>7</v>
       </c>
       <c r="AB16" t="n">
-        <v>52</v>
+        <v>624</v>
       </c>
       <c r="AC16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AD16" t="n">
-        <v>0</v>
+        <v>4.86</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>44259</v>
+        <v>44350</v>
       </c>
       <c r="B17" t="n">
-        <v>159.86</v>
+        <v>53.55</v>
       </c>
       <c r="C17" t="n">
-        <v>36.78</v>
+        <v>23.48</v>
       </c>
       <c r="D17" t="n">
-        <v>2.72</v>
+        <v>4.26</v>
       </c>
       <c r="E17" t="n">
-        <v>2212</v>
+        <v>3356</v>
       </c>
       <c r="F17" t="n">
-        <v>9.67</v>
+        <v>23.38</v>
       </c>
       <c r="G17" t="n">
-        <v>2.37</v>
+        <v>2.2</v>
       </c>
       <c r="H17" t="n">
-        <v>96398400</v>
+        <v>92908480</v>
       </c>
       <c r="I17" t="n">
-        <v>7149</v>
+        <v>7228</v>
       </c>
       <c r="J17" t="n">
-        <v>7184</v>
+        <v>8349</v>
       </c>
       <c r="K17" t="n">
-        <v>-35</v>
+        <v>-1121</v>
       </c>
       <c r="L17" t="n">
-        <v>-0</v>
+        <v>-0.11</v>
       </c>
       <c r="M17" t="n">
-        <v>-0</v>
+        <v>-0.03</v>
       </c>
       <c r="N17" t="n">
-        <v>11.11</v>
+        <v>9.19</v>
       </c>
       <c r="O17" t="n">
-        <v>6.43</v>
+        <v>9.33</v>
       </c>
       <c r="P17" t="n">
-        <v>6.37</v>
+        <v>8.99</v>
       </c>
       <c r="Q17" t="n">
-        <v>3057</v>
+        <v>3560</v>
       </c>
       <c r="R17" t="n">
-        <v>-2556</v>
+        <v>-2081</v>
       </c>
       <c r="S17" t="n">
-        <v>5</v>
+        <v>-228</v>
       </c>
       <c r="T17" t="n">
-        <v>39</v>
+        <v>1301</v>
       </c>
       <c r="U17" t="n">
-        <v>3018</v>
+        <v>2259</v>
       </c>
       <c r="V17" t="n">
-        <v>3933</v>
+        <v>3944</v>
       </c>
       <c r="W17" t="n">
-        <v>641</v>
+        <v>670</v>
       </c>
       <c r="X17" t="n">
         <v>6551</v>
       </c>
       <c r="Y17" t="n">
-        <v>11846</v>
+        <v>13099</v>
       </c>
       <c r="Z17" t="n">
-        <v>188.83</v>
+        <v>152.23</v>
       </c>
       <c r="AA17" t="n">
-        <v>258</v>
+        <v>764</v>
       </c>
       <c r="AB17" t="n">
-        <v>-275</v>
+        <v>52</v>
       </c>
       <c r="AC17" t="n">
         <v>0</v>
@@ -3130,96 +3130,191 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
+        <v>44259</v>
+      </c>
+      <c r="B18" t="n">
+        <v>159.79</v>
+      </c>
+      <c r="C18" t="n">
+        <v>36.76</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2212</v>
+      </c>
+      <c r="F18" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H18" t="n">
+        <v>96353600</v>
+      </c>
+      <c r="I18" t="n">
+        <v>7149</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7184</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-35</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3057</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-2556</v>
+      </c>
+      <c r="S18" t="n">
+        <v>5</v>
+      </c>
+      <c r="T18" t="n">
+        <v>39</v>
+      </c>
+      <c r="U18" t="n">
+        <v>3018</v>
+      </c>
+      <c r="V18" t="n">
+        <v>3933</v>
+      </c>
+      <c r="W18" t="n">
+        <v>641</v>
+      </c>
+      <c r="X18" t="n">
+        <v>6551</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>11846</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>188.83</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>258</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>-275</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>44168</v>
       </c>
-      <c r="B18" t="n">
-        <v>101.85</v>
-      </c>
-      <c r="C18" t="n">
-        <v>32.75</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="B19" t="n">
+        <v>101.81</v>
+      </c>
+      <c r="C19" t="n">
+        <v>32.73</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="E19" t="n">
         <v>2353</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F19" t="n">
         <v>13.91</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G19" t="n">
         <v>2.05</v>
       </c>
-      <c r="H18" t="n">
-        <v>81785250</v>
-      </c>
-      <c r="I18" t="n">
+      <c r="H19" t="n">
+        <v>81751799.99999999</v>
+      </c>
+      <c r="I19" t="n">
         <v>7158</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J19" t="n">
         <v>7032</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K19" t="n">
         <v>126</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L19" t="n">
         <v>0.02</v>
       </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="n">
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
         <v>9.890000000000001</v>
       </c>
-      <c r="O18" t="n">
+      <c r="O19" t="n">
         <v>6.27</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P19" t="n">
         <v>6.18</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q19" t="n">
         <v>1967</v>
       </c>
-      <c r="R18" t="n">
+      <c r="R19" t="n">
         <v>-3418</v>
       </c>
-      <c r="S18" t="n">
+      <c r="S19" t="n">
         <v>-214</v>
       </c>
-      <c r="T18" t="n">
+      <c r="T19" t="n">
         <v>-771</v>
       </c>
-      <c r="U18" t="n">
+      <c r="U19" t="n">
         <v>2738</v>
       </c>
-      <c r="V18" t="n">
+      <c r="V19" t="n">
         <v>3111</v>
       </c>
-      <c r="W18" t="n">
+      <c r="W19" t="n">
         <v>647</v>
       </c>
-      <c r="X18" t="n">
+      <c r="X19" t="n">
         <v>5728</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Y19" t="n">
         <v>10841</v>
       </c>
-      <c r="Z18" t="n">
+      <c r="Z19" t="n">
         <v>211.35</v>
       </c>
-      <c r="AA18" t="n">
+      <c r="AA19" t="n">
         <v>-395</v>
       </c>
-      <c r="AB18" t="n">
+      <c r="AB19" t="n">
         <v>-815</v>
       </c>
-      <c r="AC18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE18" t="n">
+      <c r="AC19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>